<commit_message>
Corregge griglia pranzi: Mens Sana Siena ven 14:00 → Pool Bar
Caffè Micky 14:00: 76→40 coperti · Pool Bar 14:00: 65→101 coperti
Aggiornati totali Venerdì, Riepilogo e foglio Allergie

https://claude.ai/code/session_01L71tgdEaT7WMMAgsiZmcki
</commit_message>
<xml_diff>
--- a/griglia_pranzi_torneo.xlsx
+++ b/griglia_pranzi_torneo.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riepilogo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venerdì" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sabato" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domenica" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⚠ Allergie" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Riepilogo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Venerdì" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sabato" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Domenica" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="⚠ Allergie" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Riepilogo'!$1:$3</definedName>
@@ -193,7 +193,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -229,11 +229,99 @@
         <color rgb="000A1F5C"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="000A1F5C"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="000A1F5C"/>
+      </right>
+      <top style="medium">
+        <color rgb="000A1F5C"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="000A1F5C"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000A1F5C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="000A1F5C"/>
+      </right>
+      <top style="medium">
+        <color rgb="000A1F5C"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000A1F5C"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -342,6 +430,10 @@
     <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -908,7 +1000,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Caffè Micky</t>
+          <t>Pool Bar</t>
         </is>
       </c>
       <c r="G8" s="13" t="inlineStr">
@@ -1639,6 +1731,8 @@
           <t>Allergie &amp; intolleranze (⚠ segnalare alla cucina)</t>
         </is>
       </c>
+      <c r="E5" s="40" t="n"/>
+      <c r="F5" s="41" t="n"/>
       <c r="G5" s="17" t="inlineStr">
         <is>
           <t>Confermato ✓</t>
@@ -1664,6 +1758,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="E6" s="40" t="n"/>
+      <c r="F6" s="41" t="n"/>
       <c r="G6" s="19" t="inlineStr"/>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -1672,15 +1768,19 @@
           <t>TOTALE TURNO</t>
         </is>
       </c>
+      <c r="B7" s="41" t="n"/>
       <c r="C7" s="20" t="n">
         <v>24</v>
       </c>
       <c r="D7" s="21" t="inlineStr"/>
+      <c r="E7" s="40" t="n"/>
+      <c r="F7" s="40" t="n"/>
+      <c r="G7" s="41" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ⏱ Turno ore 14:00  —  76 coperti totali  ⚠ 2 squadra/e con allergie/intolleranze</t>
+          <t xml:space="preserve">  ⏱ Turno ore 14:00  —  40 coperti totali  ⚠ 1 squadra/e con allergie/intolleranze</t>
         </is>
       </c>
     </row>
@@ -1705,6 +1805,8 @@
           <t>Allergie &amp; intolleranze (⚠ segnalare alla cucina)</t>
         </is>
       </c>
+      <c r="E9" s="40" t="n"/>
+      <c r="F9" s="41" t="n"/>
       <c r="G9" s="17" t="inlineStr">
         <is>
           <t>Confermato ✓</t>
@@ -1714,7 +1816,7 @@
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Mens Sana Siena</t>
+          <t>TissIttiri</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1723,19 +1825,21 @@
         </is>
       </c>
       <c r="C10" s="18" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>⚠ 1 celiaco</t>
-        </is>
-      </c>
+          <t>⚠ 1 allergia peperoncino rosso · 1 intolleranza lattosio · 1 allergia tonno</t>
+        </is>
+      </c>
+      <c r="E10" s="40" t="n"/>
+      <c r="F10" s="41" t="n"/>
       <c r="G10" s="19" t="inlineStr"/>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>TissIttiri</t>
+          <t>Basket Marsciano</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1744,185 +1848,210 @@
         </is>
       </c>
       <c r="C11" s="18" t="n">
-        <v>24</v>
-      </c>
-      <c r="D11" s="23" t="inlineStr">
-        <is>
-          <t>⚠ 1 allergia peperoncino rosso · 1 intolleranza lattosio · 1 allergia tonno</t>
-        </is>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="40" t="n"/>
+      <c r="F11" s="41" t="n"/>
       <c r="G11" s="19" t="inlineStr"/>
     </row>
     <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Basket Marsciano</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C12" s="18" t="n">
-        <v>16</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G12" s="19" t="inlineStr"/>
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>TOTALE TURNO</t>
+        </is>
+      </c>
+      <c r="B12" s="41" t="n"/>
+      <c r="C12" s="20" t="n">
+        <v>40</v>
+      </c>
+      <c r="D12" s="21" t="inlineStr"/>
+      <c r="E12" s="40" t="n"/>
+      <c r="F12" s="40" t="n"/>
+      <c r="G12" s="41" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>TOTALE TURNO</t>
-        </is>
-      </c>
-      <c r="C13" s="20" t="n">
-        <v>76</v>
-      </c>
-      <c r="D13" s="21" t="inlineStr"/>
-    </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>TOTALE CAFFÈ MICKY</t>
         </is>
       </c>
-      <c r="C14" s="25" t="n">
-        <v>100</v>
-      </c>
-      <c r="D14" s="26" t="inlineStr"/>
+      <c r="B13" s="42" t="n"/>
+      <c r="C13" s="25" t="n">
+        <v>64</v>
+      </c>
+      <c r="D13" s="26" t="inlineStr"/>
+      <c r="E13" s="43" t="n"/>
+      <c r="F13" s="43" t="n"/>
+      <c r="G13" s="42" t="n"/>
+    </row>
+    <row r="14" ht="28" customHeight="1"/>
+    <row r="15">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  📍 Pool Bar  —  Piazza Sandro Pertini, Monsummano Terme</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  📍 Pool Bar  —  Piazza Sandro Pertini, Monsummano Terme</t>
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⏱ Turno ore 12:30  —  25 coperti totali  ⚠ 1 squadra/e con allergie/intolleranze</t>
         </is>
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ⏱ Turno ore 12:30  —  25 coperti totali  ⚠ 1 squadra/e con allergie/intolleranze</t>
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Squadra</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Cat.</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Allergie &amp; intolleranze (⚠ segnalare alla cucina)</t>
+        </is>
+      </c>
+      <c r="E17" s="40" t="n"/>
+      <c r="F17" s="41" t="n"/>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>Confermato ✓</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Squadra</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>Cat.</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="inlineStr">
-        <is>
-          <t>PAX</t>
-        </is>
-      </c>
-      <c r="D18" s="17" t="inlineStr">
-        <is>
-          <t>Allergie &amp; intolleranze (⚠ segnalare alla cucina)</t>
-        </is>
-      </c>
-      <c r="G18" s="17" t="inlineStr">
-        <is>
-          <t>Confermato ✓</t>
-        </is>
-      </c>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Chiesina Basket</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
+        </is>
+      </c>
+      <c r="E18" s="40" t="n"/>
+      <c r="F18" s="41" t="n"/>
+      <c r="G18" s="19" t="inlineStr"/>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Chiesina Basket</t>
+          <t>Dany Basket</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="C19" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="D19" s="23" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" s="40" t="n"/>
+      <c r="F19" s="41" t="n"/>
       <c r="G19" s="19" t="inlineStr"/>
     </row>
     <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Dany Basket</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>TOTALE TURNO</t>
+        </is>
+      </c>
+      <c r="B20" s="41" t="n"/>
+      <c r="C20" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="D20" s="21" t="inlineStr"/>
+      <c r="E20" s="40" t="n"/>
+      <c r="F20" s="40" t="n"/>
+      <c r="G20" s="41" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⏱ Turno ore 14:00  —  101 coperti totali  ⚠ 2 squadra/e con allergie/intolleranze</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Squadra</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>Cat.</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>PAX</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>Allergie &amp; intolleranze (⚠ segnalare alla cucina)</t>
+        </is>
+      </c>
+      <c r="E22" s="40" t="n"/>
+      <c r="F22" s="41" t="n"/>
+      <c r="G22" s="17" t="inlineStr">
+        <is>
+          <t>Confermato ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Mens Sana Siena</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>U13</t>
         </is>
       </c>
-      <c r="C20" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G20" s="19" t="inlineStr"/>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
-        <is>
-          <t>TOTALE TURNO</t>
-        </is>
-      </c>
-      <c r="C21" s="20" t="n">
-        <v>25</v>
-      </c>
-      <c r="D21" s="21" t="inlineStr"/>
-    </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ⏱ Turno ore 14:00  —  65 coperti totali  ⚠ 1 squadra/e con allergie/intolleranze</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
-        <is>
-          <t>Squadra</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>Cat.</t>
-        </is>
-      </c>
-      <c r="C23" s="17" t="inlineStr">
-        <is>
-          <t>PAX</t>
-        </is>
-      </c>
-      <c r="D23" s="17" t="inlineStr">
-        <is>
-          <t>Allergie &amp; intolleranze (⚠ segnalare alla cucina)</t>
-        </is>
-      </c>
-      <c r="G23" s="17" t="inlineStr">
-        <is>
-          <t>Confermato ✓</t>
-        </is>
-      </c>
+      <c r="C23" s="18" t="n">
+        <v>36</v>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco</t>
+        </is>
+      </c>
+      <c r="E23" s="40" t="n"/>
+      <c r="F23" s="41" t="n"/>
+      <c r="G23" s="19" t="n"/>
     </row>
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
@@ -1943,6 +2072,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="E24" s="40" t="n"/>
+      <c r="F24" s="41" t="n"/>
       <c r="G24" s="19" t="inlineStr"/>
     </row>
     <row r="25" ht="26" customHeight="1">
@@ -1964,6 +2095,8 @@
           <t>⚠ 1 celiaco</t>
         </is>
       </c>
+      <c r="E25" s="40" t="n"/>
+      <c r="F25" s="41" t="n"/>
       <c r="G25" s="19" t="inlineStr"/>
     </row>
     <row r="26" ht="26" customHeight="1">
@@ -1985,6 +2118,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="E26" s="40" t="n"/>
+      <c r="F26" s="41" t="n"/>
       <c r="G26" s="19" t="inlineStr"/>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -1993,10 +2128,14 @@
           <t>TOTALE TURNO</t>
         </is>
       </c>
+      <c r="B27" s="41" t="n"/>
       <c r="C27" s="20" t="n">
-        <v>65</v>
+        <v>101</v>
       </c>
       <c r="D27" s="21" t="inlineStr"/>
+      <c r="E27" s="40" t="n"/>
+      <c r="F27" s="40" t="n"/>
+      <c r="G27" s="41" t="n"/>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="28" t="inlineStr">
@@ -2004,11 +2143,16 @@
           <t>TOTALE POOL BAR</t>
         </is>
       </c>
+      <c r="B28" s="42" t="n"/>
       <c r="C28" s="29" t="n">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="D28" s="30" t="inlineStr"/>
-    </row>
+      <c r="E28" s="43" t="n"/>
+      <c r="F28" s="43" t="n"/>
+      <c r="G28" s="42" t="n"/>
+    </row>
+    <row r="29"/>
     <row r="30" ht="26" customHeight="1">
       <c r="A30" s="31" t="inlineStr">
         <is>
@@ -2022,10 +2166,14 @@
           <t xml:space="preserve">  Pool Bar</t>
         </is>
       </c>
+      <c r="B31" s="41" t="n"/>
       <c r="C31" s="20" t="n">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="D31" s="33" t="inlineStr"/>
+      <c r="E31" s="40" t="n"/>
+      <c r="F31" s="40" t="n"/>
+      <c r="G31" s="41" t="n"/>
     </row>
     <row r="32" ht="26" customHeight="1">
       <c r="A32" s="34" t="inlineStr">
@@ -2033,10 +2181,14 @@
           <t xml:space="preserve">  Caffè Micky</t>
         </is>
       </c>
+      <c r="B32" s="41" t="n"/>
       <c r="C32" s="20" t="n">
-        <v>100</v>
+        <v>64</v>
       </c>
       <c r="D32" s="33" t="inlineStr"/>
+      <c r="E32" s="40" t="n"/>
+      <c r="F32" s="40" t="n"/>
+      <c r="G32" s="41" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="35" t="inlineStr">
@@ -2044,10 +2196,14 @@
           <t xml:space="preserve">  TOTALE COPERTI</t>
         </is>
       </c>
+      <c r="B33" s="42" t="n"/>
       <c r="C33" s="36" t="n">
         <v>190</v>
       </c>
       <c r="D33" s="37" t="inlineStr"/>
+      <c r="E33" s="43" t="n"/>
+      <c r="F33" s="43" t="n"/>
+      <c r="G33" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="40">
@@ -2162,6 +2318,8 @@
           <t>Allergie &amp; intolleranze (⚠ segnalare alla cucina)</t>
         </is>
       </c>
+      <c r="E5" s="40" t="n"/>
+      <c r="F5" s="41" t="n"/>
       <c r="G5" s="17" t="inlineStr">
         <is>
           <t>Confermato ✓</t>
@@ -2187,6 +2345,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="E6" s="40" t="n"/>
+      <c r="F6" s="41" t="n"/>
       <c r="G6" s="19" t="inlineStr"/>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -2195,10 +2355,14 @@
           <t>TOTALE TURNO</t>
         </is>
       </c>
+      <c r="B7" s="41" t="n"/>
       <c r="C7" s="20" t="n">
         <v>16</v>
       </c>
       <c r="D7" s="21" t="inlineStr"/>
+      <c r="E7" s="40" t="n"/>
+      <c r="F7" s="40" t="n"/>
+      <c r="G7" s="41" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="22" t="inlineStr">
@@ -2228,6 +2392,8 @@
           <t>Allergie &amp; intolleranze (⚠ segnalare alla cucina)</t>
         </is>
       </c>
+      <c r="E9" s="40" t="n"/>
+      <c r="F9" s="41" t="n"/>
       <c r="G9" s="17" t="inlineStr">
         <is>
           <t>Confermato ✓</t>
@@ -2253,6 +2419,8 @@
           <t>⚠ 1 celiaco</t>
         </is>
       </c>
+      <c r="E10" s="40" t="n"/>
+      <c r="F10" s="41" t="n"/>
       <c r="G10" s="19" t="inlineStr"/>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -2261,10 +2429,14 @@
           <t>TOTALE TURNO</t>
         </is>
       </c>
+      <c r="B11" s="41" t="n"/>
       <c r="C11" s="20" t="n">
         <v>4</v>
       </c>
       <c r="D11" s="21" t="inlineStr"/>
+      <c r="E11" s="40" t="n"/>
+      <c r="F11" s="40" t="n"/>
+      <c r="G11" s="41" t="n"/>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
@@ -2272,10 +2444,14 @@
           <t>TOTALE CAFFÈ MICKY</t>
         </is>
       </c>
+      <c r="B12" s="42" t="n"/>
       <c r="C12" s="25" t="n">
         <v>20</v>
       </c>
       <c r="D12" s="26" t="inlineStr"/>
+      <c r="E12" s="43" t="n"/>
+      <c r="F12" s="43" t="n"/>
+      <c r="G12" s="42" t="n"/>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="27" t="inlineStr">
@@ -2312,6 +2488,8 @@
           <t>Allergie &amp; intolleranze (⚠ segnalare alla cucina)</t>
         </is>
       </c>
+      <c r="E16" s="40" t="n"/>
+      <c r="F16" s="41" t="n"/>
       <c r="G16" s="17" t="inlineStr">
         <is>
           <t>Confermato ✓</t>
@@ -2337,6 +2515,8 @@
           <t>⚠ 1 allergia peperoncino rosso · 1 intolleranza lattosio · 1 allergia tonno</t>
         </is>
       </c>
+      <c r="E17" s="40" t="n"/>
+      <c r="F17" s="41" t="n"/>
       <c r="G17" s="19" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
@@ -2345,10 +2525,14 @@
           <t>TOTALE TURNO</t>
         </is>
       </c>
+      <c r="B18" s="41" t="n"/>
       <c r="C18" s="20" t="n">
         <v>24</v>
       </c>
       <c r="D18" s="21" t="inlineStr"/>
+      <c r="E18" s="40" t="n"/>
+      <c r="F18" s="40" t="n"/>
+      <c r="G18" s="41" t="n"/>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="22" t="inlineStr">
@@ -2378,6 +2562,8 @@
           <t>Allergie &amp; intolleranze (⚠ segnalare alla cucina)</t>
         </is>
       </c>
+      <c r="E20" s="40" t="n"/>
+      <c r="F20" s="41" t="n"/>
       <c r="G20" s="17" t="inlineStr">
         <is>
           <t>Confermato ✓</t>
@@ -2403,6 +2589,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="E21" s="40" t="n"/>
+      <c r="F21" s="41" t="n"/>
       <c r="G21" s="19" t="inlineStr"/>
     </row>
     <row r="22" ht="26" customHeight="1">
@@ -2424,6 +2612,8 @@
           <t>⚠ 1 celiaco</t>
         </is>
       </c>
+      <c r="E22" s="40" t="n"/>
+      <c r="F22" s="41" t="n"/>
       <c r="G22" s="19" t="inlineStr"/>
     </row>
     <row r="23" ht="26" customHeight="1">
@@ -2445,6 +2635,8 @@
           <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
         </is>
       </c>
+      <c r="E23" s="40" t="n"/>
+      <c r="F23" s="41" t="n"/>
       <c r="G23" s="19" t="inlineStr"/>
     </row>
     <row r="24" ht="26" customHeight="1">
@@ -2466,6 +2658,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="E24" s="40" t="n"/>
+      <c r="F24" s="41" t="n"/>
       <c r="G24" s="19" t="inlineStr"/>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -2474,10 +2668,14 @@
           <t>TOTALE TURNO</t>
         </is>
       </c>
+      <c r="B25" s="41" t="n"/>
       <c r="C25" s="20" t="n">
         <v>80</v>
       </c>
       <c r="D25" s="21" t="inlineStr"/>
+      <c r="E25" s="40" t="n"/>
+      <c r="F25" s="40" t="n"/>
+      <c r="G25" s="41" t="n"/>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="28" t="inlineStr">
@@ -2485,10 +2683,14 @@
           <t>TOTALE POOL BAR</t>
         </is>
       </c>
+      <c r="B26" s="42" t="n"/>
       <c r="C26" s="29" t="n">
         <v>104</v>
       </c>
       <c r="D26" s="30" t="inlineStr"/>
+      <c r="E26" s="43" t="n"/>
+      <c r="F26" s="43" t="n"/>
+      <c r="G26" s="42" t="n"/>
     </row>
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="31" t="inlineStr">
@@ -2503,10 +2705,14 @@
           <t xml:space="preserve">  Pool Bar</t>
         </is>
       </c>
+      <c r="B29" s="41" t="n"/>
       <c r="C29" s="20" t="n">
         <v>104</v>
       </c>
       <c r="D29" s="33" t="inlineStr"/>
+      <c r="E29" s="40" t="n"/>
+      <c r="F29" s="40" t="n"/>
+      <c r="G29" s="41" t="n"/>
     </row>
     <row r="30" ht="26" customHeight="1">
       <c r="A30" s="34" t="inlineStr">
@@ -2514,10 +2720,14 @@
           <t xml:space="preserve">  Caffè Micky</t>
         </is>
       </c>
+      <c r="B30" s="41" t="n"/>
       <c r="C30" s="20" t="n">
         <v>20</v>
       </c>
       <c r="D30" s="33" t="inlineStr"/>
+      <c r="E30" s="40" t="n"/>
+      <c r="F30" s="40" t="n"/>
+      <c r="G30" s="41" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="35" t="inlineStr">
@@ -2525,10 +2735,14 @@
           <t xml:space="preserve">  TOTALE COPERTI</t>
         </is>
       </c>
+      <c r="B31" s="42" t="n"/>
       <c r="C31" s="36" t="n">
         <v>124</v>
       </c>
       <c r="D31" s="37" t="inlineStr"/>
+      <c r="E31" s="43" t="n"/>
+      <c r="F31" s="43" t="n"/>
+      <c r="G31" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="38">
@@ -2641,6 +2855,8 @@
           <t>Allergie &amp; intolleranze (⚠ segnalare alla cucina)</t>
         </is>
       </c>
+      <c r="E5" s="40" t="n"/>
+      <c r="F5" s="41" t="n"/>
       <c r="G5" s="17" t="inlineStr">
         <is>
           <t>Confermato ✓</t>
@@ -2666,6 +2882,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="E6" s="40" t="n"/>
+      <c r="F6" s="41" t="n"/>
       <c r="G6" s="19" t="inlineStr"/>
     </row>
     <row r="7" ht="26" customHeight="1">
@@ -2687,6 +2905,8 @@
           <t>⚠ 1 allergia peperoncino rosso · 1 intolleranza lattosio · 1 allergia tonno</t>
         </is>
       </c>
+      <c r="E7" s="40" t="n"/>
+      <c r="F7" s="41" t="n"/>
       <c r="G7" s="19" t="inlineStr"/>
     </row>
     <row r="8" ht="26" customHeight="1">
@@ -2708,6 +2928,8 @@
           <t>⚠ 1 celiaco</t>
         </is>
       </c>
+      <c r="E8" s="40" t="n"/>
+      <c r="F8" s="41" t="n"/>
       <c r="G8" s="19" t="inlineStr"/>
     </row>
     <row r="9" ht="26" customHeight="1">
@@ -2729,6 +2951,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="E9" s="40" t="n"/>
+      <c r="F9" s="41" t="n"/>
       <c r="G9" s="19" t="inlineStr"/>
     </row>
     <row r="10" ht="26" customHeight="1">
@@ -2750,6 +2974,8 @@
           <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
         </is>
       </c>
+      <c r="E10" s="40" t="n"/>
+      <c r="F10" s="41" t="n"/>
       <c r="G10" s="19" t="inlineStr"/>
     </row>
     <row r="11" ht="26" customHeight="1">
@@ -2771,6 +2997,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="E11" s="40" t="n"/>
+      <c r="F11" s="41" t="n"/>
       <c r="G11" s="19" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -2779,10 +3007,14 @@
           <t>TOTALE TURNO</t>
         </is>
       </c>
+      <c r="B12" s="41" t="n"/>
       <c r="C12" s="20" t="n">
         <v>120</v>
       </c>
       <c r="D12" s="21" t="inlineStr"/>
+      <c r="E12" s="40" t="n"/>
+      <c r="F12" s="40" t="n"/>
+      <c r="G12" s="41" t="n"/>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="28" t="inlineStr">
@@ -2790,10 +3022,14 @@
           <t>TOTALE POOL BAR</t>
         </is>
       </c>
+      <c r="B13" s="42" t="n"/>
       <c r="C13" s="29" t="n">
         <v>120</v>
       </c>
       <c r="D13" s="30" t="inlineStr"/>
+      <c r="E13" s="43" t="n"/>
+      <c r="F13" s="43" t="n"/>
+      <c r="G13" s="42" t="n"/>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="31" t="inlineStr">
@@ -2808,10 +3044,14 @@
           <t xml:space="preserve">  Pool Bar</t>
         </is>
       </c>
+      <c r="B16" s="41" t="n"/>
       <c r="C16" s="20" t="n">
         <v>120</v>
       </c>
       <c r="D16" s="33" t="inlineStr"/>
+      <c r="E16" s="40" t="n"/>
+      <c r="F16" s="40" t="n"/>
+      <c r="G16" s="41" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="35" t="inlineStr">
@@ -2819,10 +3059,14 @@
           <t xml:space="preserve">  TOTALE COPERTI</t>
         </is>
       </c>
+      <c r="B17" s="42" t="n"/>
       <c r="C17" s="36" t="n">
         <v>120</v>
       </c>
       <c r="D17" s="37" t="inlineStr"/>
+      <c r="E17" s="43" t="n"/>
+      <c r="F17" s="43" t="n"/>
+      <c r="G17" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="20">
@@ -3002,7 +3246,7 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Caffè Micky</t>
+          <t>Pool Bar</t>
         </is>
       </c>
       <c r="F6" s="23" t="inlineStr">

</xml_diff>

<commit_message>
Nasconde sezione Domenica dalla griglia pranzi (da confermare)
https://claude.ai/code/session_01L71tgdEaT7WMMAgsiZmcki
</commit_message>
<xml_diff>
--- a/griglia_pranzi_torneo.xlsx
+++ b/griglia_pranzi_torneo.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Riepilogo" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Venerdì" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Sabato" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Domenica" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Domenica" sheetId="4" state="hidden" r:id="rId4"/>
     <sheet name="⚠ Allergie" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
@@ -1436,14 +1436,14 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="24" customHeight="1">
+    <row r="22" hidden="1" ht="24" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  DOMENICA 3 MAGGIO</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="28" customHeight="1">
+    <row r="23" hidden="1" ht="28" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>TissIttiri</t>
@@ -1478,7 +1478,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="28" customHeight="1">
+    <row r="24" hidden="1" ht="28" customHeight="1">
       <c r="A24" s="10" t="inlineStr">
         <is>
           <t>San Fr. Ittiri</t>
@@ -1513,7 +1513,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" hidden="1" ht="28" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Basket Marsciano</t>
@@ -1548,7 +1548,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="28" customHeight="1">
+    <row r="26" hidden="1" ht="28" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Codigoro Basket</t>
@@ -1583,7 +1583,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="28" customHeight="1">
+    <row r="27" hidden="1" ht="28" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Basket Loano</t>
@@ -1618,7 +1618,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1">
+    <row r="28" hidden="1" ht="28" customHeight="1">
       <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Chiesina Basket</t>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="D12" s="21" t="inlineStr"/>
       <c r="E12" s="40" t="n"/>
-      <c r="F12" s="40" t="n"/>
+      <c r="F12" s="41" t="n"/>
       <c r="G12" s="41" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -1910,28 +1910,12 @@
           <t>Squadra</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>Cat.</t>
-        </is>
-      </c>
-      <c r="C17" s="17" t="inlineStr">
-        <is>
-          <t>PAX</t>
-        </is>
-      </c>
-      <c r="D17" s="17" t="inlineStr">
-        <is>
-          <t>Allergie &amp; intolleranze (⚠ segnalare alla cucina)</t>
-        </is>
-      </c>
+      <c r="B17" s="40" t="n"/>
+      <c r="C17" s="40" t="n"/>
+      <c r="D17" s="40" t="n"/>
       <c r="E17" s="40" t="n"/>
-      <c r="F17" s="41" t="n"/>
-      <c r="G17" s="17" t="inlineStr">
-        <is>
-          <t>Confermato ✓</t>
-        </is>
-      </c>
+      <c r="F17" s="40" t="n"/>
+      <c r="G17" s="41" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -1991,7 +1975,7 @@
       </c>
       <c r="D20" s="21" t="inlineStr"/>
       <c r="E20" s="40" t="n"/>
-      <c r="F20" s="40" t="n"/>
+      <c r="F20" s="41" t="n"/>
       <c r="G20" s="41" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
@@ -2007,28 +1991,12 @@
           <t>Squadra</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
-        <is>
-          <t>Cat.</t>
-        </is>
-      </c>
-      <c r="C22" s="17" t="inlineStr">
-        <is>
-          <t>PAX</t>
-        </is>
-      </c>
-      <c r="D22" s="17" t="inlineStr">
-        <is>
-          <t>Allergie &amp; intolleranze (⚠ segnalare alla cucina)</t>
-        </is>
-      </c>
+      <c r="B22" s="40" t="n"/>
+      <c r="C22" s="40" t="n"/>
+      <c r="D22" s="40" t="n"/>
       <c r="E22" s="40" t="n"/>
-      <c r="F22" s="41" t="n"/>
-      <c r="G22" s="17" t="inlineStr">
-        <is>
-          <t>Confermato ✓</t>
-        </is>
-      </c>
+      <c r="F22" s="40" t="n"/>
+      <c r="G22" s="41" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -2152,7 +2120,6 @@
       <c r="F28" s="43" t="n"/>
       <c r="G28" s="42" t="n"/>
     </row>
-    <row r="29"/>
     <row r="30" ht="26" customHeight="1">
       <c r="A30" s="31" t="inlineStr">
         <is>
@@ -3415,7 +3382,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" hidden="1" ht="28" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>TissIttiri</t>
@@ -3447,7 +3414,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" hidden="1" ht="28" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Basket Loano</t>
@@ -3479,7 +3446,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" hidden="1" ht="28" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Chiesina Basket</t>

</xml_diff>

<commit_message>
Aggiorna Dany Basket a 17 pax (sab 12:30 Pool Bar)
https://claude.ai/code/session_01L71tgdEaT7WMMAgsiZmcki
</commit_message>
<xml_diff>
--- a/griglia_pranzi_torneo.xlsx
+++ b/griglia_pranzi_torneo.xlsx
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="F7" s="7" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G7" s="8" t="inlineStr"/>
     </row>
@@ -1289,7 +1289,7 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🍽 Pool Bar · 12:30 · 25 coperti · ⚠ allergie</t>
+          <t xml:space="preserve">  🍽 Pool Bar · 12:30 · 32 coperti · ⚠ allergie</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="E10" s="12" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F10" s="13" t="inlineStr"/>
     </row>
@@ -1356,7 +1356,7 @@
         </is>
       </c>
       <c r="E11" s="15" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Aggiorna Dany Basket a 23 pax (sab 12:30 Pool Bar)
https://claude.ai/code/session_01L71tgdEaT7WMMAgsiZmcki
</commit_message>
<xml_diff>
--- a/griglia_pranzi_torneo.xlsx
+++ b/griglia_pranzi_torneo.xlsx
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="F7" s="7" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="G7" s="8" t="inlineStr"/>
     </row>
@@ -1289,7 +1289,7 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🍽 Pool Bar · 12:30 · 32 coperti · ⚠ allergie</t>
+          <t xml:space="preserve">  🍽 Pool Bar · 12:30 · 38 coperti · ⚠ allergie</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="E10" s="12" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F10" s="13" t="inlineStr"/>
     </row>
@@ -1356,7 +1356,7 @@
         </is>
       </c>
       <c r="E11" s="15" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Aggiorna Dany Basket: ven 27 pax (Pool Bar 12:30), sab 31 pax (Caffè Micky 13:30)
https://claude.ai/code/session_01L71tgdEaT7WMMAgsiZmcki
</commit_message>
<xml_diff>
--- a/griglia_pranzi_torneo.xlsx
+++ b/griglia_pranzi_torneo.xlsx
@@ -578,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="F7" s="7" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G7" s="8" t="inlineStr"/>
     </row>
@@ -1045,19 +1045,19 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Sabato 2 Mag</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Pool Bar</t>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Caffè Micky</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1065,15 +1065,15 @@
           <t>U13</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Codigoro Basket</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="G18" s="8" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Dany Basket</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1091,24 +1091,20 @@
           <t>Pool Bar</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>U14</t>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Basket Loano</t>
+          <t>Codigoro Basket</t>
         </is>
       </c>
       <c r="F19" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="G19" s="10" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="G19" s="8" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1133,15 +1129,15 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Chiesina Basket</t>
+          <t>Basket Loano</t>
         </is>
       </c>
       <c r="F20" s="7" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
+          <t>⚠ 1 celiaco</t>
         </is>
       </c>
     </row>
@@ -1168,13 +1164,48 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
+          <t>Chiesina Basket</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Sabato 2 Mag</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Pool Bar</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
           <t>San Fr. Ittiri</t>
         </is>
       </c>
-      <c r="F21" s="7" t="n">
+      <c r="F22" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="G21" s="8" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1289,7 +1320,7 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🍽 Pool Bar · 12:30 · 38 coperti · ⚠ allergie</t>
+          <t xml:space="preserve">  🍽 Pool Bar · 12:30 · 42 coperti · ⚠ allergie</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1376,7 @@
         </is>
       </c>
       <c r="E10" s="12" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F10" s="13" t="inlineStr"/>
     </row>
@@ -1356,7 +1387,7 @@
         </is>
       </c>
       <c r="E11" s="15" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
@@ -1598,7 +1629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1747,7 +1778,7 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ☕ Caffè Micky · 13:30 · 4 coperti · ⚠ allergie</t>
+          <t xml:space="preserve">  ☕ Caffè Micky · 13:30 · 35 coperti · ⚠ allergie</t>
         </is>
       </c>
     </row>
@@ -1782,52 +1813,52 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Caffè Micky</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Dany Basket</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="F14" s="13" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>TOTALE COPERTI</t>
         </is>
       </c>
-      <c r="E14" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="E15" s="15" t="n">
+        <v>35</v>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
         <is>
           <t>⚠ allergie presenti</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  🍽 Pool Bar · 13:30 · 80 coperti · ⚠ allergie</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>Pool Bar</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Codigoro Basket</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="n">
-        <v>35</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -1840,24 +1871,20 @@
           <t>Pool Bar</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>U14</t>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Basket Loano</t>
+          <t>Codigoro Basket</t>
         </is>
       </c>
       <c r="E18" s="12" t="n">
-        <v>18</v>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -1877,15 +1904,15 @@
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>Chiesina Basket</t>
+          <t>Basket Loano</t>
         </is>
       </c>
       <c r="E19" s="12" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
+          <t>⚠ 1 celiaco</t>
         </is>
       </c>
     </row>
@@ -1907,24 +1934,54 @@
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
+          <t>Chiesina Basket</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Pool Bar</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
           <t>San Fr. Ittiri</t>
         </is>
       </c>
-      <c r="E20" s="12" t="n">
+      <c r="E21" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="F20" s="13" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="F21" s="13" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>TOTALE COPERTI</t>
         </is>
       </c>
-      <c r="E21" s="15" t="n">
+      <c r="E22" s="15" t="n">
         <v>80</v>
       </c>
-      <c r="F21" s="18" t="inlineStr">
+      <c r="F22" s="18" t="inlineStr">
         <is>
           <t>⚠ allergie presenti</t>
         </is>
@@ -1932,15 +1989,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A22:D22"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A21:D21"/>
     <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aggiunge Shoemakers e La T Gema alla mensa venerdì
- Shoemakers U13 9 pax · Caffè Micky 12:30 (tot. 33)
- Shoemakers U14 9 pax · Pool Bar 14:00 (tot. 121)
- La T Gema U14 11 pax · Pool Bar 14:00

https://claude.ai/code/session_01L71tgdEaT7WMMAgsiZmcki
</commit_message>
<xml_diff>
--- a/griglia_pranzi_torneo.xlsx
+++ b/griglia_pranzi_torneo.xlsx
@@ -578,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -673,39 +673,35 @@
       <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Venerdì 1 Mag</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Pool Bar</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Chiesina Basket</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
-        </is>
-      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Caffè Micky</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Shoemakers</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -723,55 +719,55 @@
           <t>Pool Bar</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>U13</t>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>U14</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
+          <t>Chiesina Basket</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Venerdì 1 Mag</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Pool Bar</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
           <t>Dany Basket</t>
         </is>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F8" s="7" t="n">
         <v>27</v>
       </c>
-      <c r="G7" s="8" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Venerdì 1 Mag</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Caffè Micky</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>TissIttiri</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
-        </is>
-      </c>
+      <c r="G8" s="8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -796,48 +792,48 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
+          <t>TissIttiri</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Venerdì 1 Mag</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Caffè Micky</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
           <t>Basket Marsciano</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F10" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Venerdì 1 Mag</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Pool Bar</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>Mens Sana Siena</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>36</v>
-      </c>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco</t>
-        </is>
-      </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -862,13 +858,17 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Codigoro Basket</t>
+          <t>Mens Sana Siena</t>
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="G11" s="8" t="inlineStr"/>
+        <v>36</v>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -886,24 +886,20 @@
           <t>Pool Bar</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>U14</t>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Basket Loano</t>
+          <t>Codigoro Basket</t>
         </is>
       </c>
       <c r="F12" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="G12" s="8" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -928,61 +924,89 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
+          <t>Basket Loano</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Venerdì 1 Mag</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Pool Bar</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
           <t>San Fr. Ittiri</t>
         </is>
       </c>
-      <c r="F13" s="7" t="n">
+      <c r="F14" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="G13" s="8" t="inlineStr"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  GIORNO 2 — Sabato 2 Maggio</t>
-        </is>
-      </c>
+      <c r="G14" s="8" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Sabato 2 Mag</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Caffè Micky</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Basket Marsciano</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="G15" s="5" t="inlineStr"/>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Venerdì 1 Mag</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Pool Bar</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Shoemakers</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="G15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Sabato 2 Mag</t>
+          <t>Venerdì 1 Mag</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -990,57 +1014,25 @@
           <t>Pool Bar</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>U13</t>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>U14</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>TissIttiri</t>
+          <t>La T Gema</t>
         </is>
       </c>
       <c r="F16" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Sabato 2 Mag</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Caffè Micky</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Mens Sana Siena</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco</t>
+        <v>11</v>
+      </c>
+      <c r="G16" s="8" t="inlineStr"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GIORNO 2 — Sabato 2 Maggio</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1044,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -1067,11 +1059,11 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Dany Basket</t>
+          <t>Basket Marsciano</t>
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G18" s="5" t="inlineStr"/>
     </row>
@@ -1083,98 +1075,98 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Pool Bar</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>TissIttiri</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sabato 2 Mag</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Pool Bar</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Codigoro Basket</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="G19" s="8" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Caffè Micky</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Mens Sana Siena</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Sabato 2 Mag</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Pool Bar</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Basket Loano</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Sabato 2 Mag</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Pool Bar</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>Chiesina Basket</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="G21" s="10" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
-        </is>
-      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Caffè Micky</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Dany Basket</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="G21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1192,25 +1184,126 @@
           <t>Pool Bar</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Codigoro Basket</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="G22" s="8" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Sabato 2 Mag</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Pool Bar</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>U14</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Basket Loano</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Sabato 2 Mag</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Pool Bar</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Chiesina Basket</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Sabato 2 Mag</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Pool Bar</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>San Fr. Ittiri</t>
         </is>
       </c>
-      <c r="F22" s="7" t="n">
+      <c r="F25" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="G22" s="8" t="inlineStr"/>
+      <c r="G25" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A14:G14"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
     <mergeCell ref="A4:G4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1223,7 +1316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1276,7 +1369,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ☕ Caffè Micky · 12:30 · 24 coperti</t>
+          <t xml:space="preserve">  ☕ Caffè Micky · 12:30 · 33 coperti</t>
         </is>
       </c>
     </row>
@@ -1307,50 +1400,46 @@
       <c r="F5" s="13" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Caffè Micky</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Shoemakers</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>TOTALE COPERTI</t>
         </is>
       </c>
-      <c r="E6" s="15" t="n">
-        <v>24</v>
-      </c>
-      <c r="F6" s="16" t="inlineStr"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="E7" s="15" t="n">
+        <v>33</v>
+      </c>
+      <c r="F7" s="16" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  🍽 Pool Bar · 12:30 · 42 coperti · ⚠ allergie</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Pool Bar</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Chiesina Basket</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="n">
-        <v>15</v>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
         </is>
       </c>
     </row>
@@ -1365,70 +1454,70 @@
           <t>Pool Bar</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>U13</t>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>U14</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
+          <t>Chiesina Basket</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Pool Bar</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
           <t>Dany Basket</t>
         </is>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E11" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="F10" s="13" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>TOTALE COPERTI</t>
         </is>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E12" s="15" t="n">
         <v>42</v>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F12" s="18" t="inlineStr">
         <is>
           <t>⚠ allergie presenti</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  ☕ Caffè Micky · 14:00 · 40 coperti · ⚠ allergie</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Caffè Micky</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>TissIttiri</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="n">
-        <v>24</v>
-      </c>
-      <c r="F14" s="10" t="inlineStr">
-        <is>
-          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
         </is>
       </c>
     </row>
@@ -1450,63 +1539,63 @@
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
+          <t>TissIttiri</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Caffè Micky</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
           <t>Basket Marsciano</t>
         </is>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E16" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="F15" s="13" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>TOTALE COPERTI</t>
         </is>
       </c>
-      <c r="E16" s="15" t="n">
+      <c r="E17" s="15" t="n">
         <v>40</v>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F17" s="18" t="inlineStr">
         <is>
           <t>⚠ allergie presenti</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🍽 Pool Bar · 14:00 · 101 coperti · ⚠ allergie</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="B19" s="13" t="inlineStr">
-        <is>
-          <t>Pool Bar</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
-        <is>
-          <t>Mens Sana Siena</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="n">
-        <v>36</v>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco</t>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🍽 Pool Bar · 14:00 · 121 coperti · ⚠ allergie</t>
         </is>
       </c>
     </row>
@@ -1528,13 +1617,17 @@
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>Codigoro Basket</t>
+          <t>Mens Sana Siena</t>
         </is>
       </c>
       <c r="E20" s="12" t="n">
-        <v>35</v>
-      </c>
-      <c r="F20" s="13" t="inlineStr"/>
+        <v>36</v>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
@@ -1547,24 +1640,20 @@
           <t>Pool Bar</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>U14</t>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>U13</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>Basket Loano</t>
+          <t>Codigoro Basket</t>
         </is>
       </c>
       <c r="E21" s="12" t="n">
-        <v>18</v>
-      </c>
-      <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="F21" s="13" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
@@ -1584,24 +1673,106 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
+          <t>Basket Loano</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Pool Bar</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
           <t>San Fr. Ittiri</t>
         </is>
       </c>
-      <c r="E22" s="12" t="n">
+      <c r="E23" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="F22" s="13" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="F23" s="13" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Pool Bar</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>Shoemakers</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Pool Bar</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>La T Gema</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="F25" s="13" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>TOTALE COPERTI</t>
         </is>
       </c>
-      <c r="E23" s="15" t="n">
-        <v>101</v>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
+      <c r="E26" s="15" t="n">
+        <v>121</v>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
         <is>
           <t>⚠ allergie presenti</t>
         </is>
@@ -1609,15 +1780,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A7:D7"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A16:D16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Rigenerazione automatica HTML ed Excel
</commit_message>
<xml_diff>
--- a/griglia_pranzi_torneo.xlsx
+++ b/griglia_pranzi_torneo.xlsx
@@ -1090,17 +1090,13 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>TissIttiri</t>
+          <t>Codigoro Basket</t>
         </is>
       </c>
       <c r="F19" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="G19" s="10" t="inlineStr">
-        <is>
-          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="G19" s="8" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1191,13 +1187,17 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Codigoro Basket</t>
+          <t>TissIttiri</t>
         </is>
       </c>
       <c r="F22" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="G22" s="8" t="inlineStr"/>
+        <v>24</v>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1897,7 +1897,7 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🍽 Pool Bar · 12:30 · 24 coperti · ⚠ allergie</t>
+          <t xml:space="preserve">  🍽 Pool Bar · 12:30 · 35 coperti</t>
         </is>
       </c>
     </row>
@@ -1919,17 +1919,13 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>TissIttiri</t>
+          <t>Codigoro Basket</t>
         </is>
       </c>
       <c r="E9" s="12" t="n">
-        <v>24</v>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -1938,13 +1934,9 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>24</v>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>⚠ allergie presenti</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="F10" s="16" t="inlineStr"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
@@ -2027,7 +2019,7 @@
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🍽 Pool Bar · 13:30 · 80 coperti · ⚠ allergie</t>
+          <t xml:space="preserve">  🍽 Pool Bar · 13:30 · 69 coperti · ⚠ allergie</t>
         </is>
       </c>
     </row>
@@ -2049,13 +2041,17 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Codigoro Basket</t>
+          <t>TissIttiri</t>
         </is>
       </c>
       <c r="E18" s="12" t="n">
-        <v>35</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr"/>
+        <v>24</v>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -2150,7 +2146,7 @@
         </is>
       </c>
       <c r="E22" s="15" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="F22" s="18" t="inlineStr">
         <is>
@@ -2384,12 +2380,12 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C8" s="21" t="inlineStr">
         <is>
-          <t>Pool Bar</t>
+          <t>Caffè Micky</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -2399,15 +2395,15 @@
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
-          <t>TissIttiri</t>
+          <t>Mens Sana Siena</t>
         </is>
       </c>
       <c r="F8" s="20" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
+          <t>⚠ 1 celiaco</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2420,7 @@
       </c>
       <c r="C9" s="21" t="inlineStr">
         <is>
-          <t>Caffè Micky</t>
+          <t>Pool Bar</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -2434,15 +2430,15 @@
       </c>
       <c r="E9" s="21" t="inlineStr">
         <is>
-          <t>Mens Sana Siena</t>
+          <t>TissIttiri</t>
         </is>
       </c>
       <c r="F9" s="20" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>⚠ 1 celiaco</t>
+          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
         </is>
       </c>
     </row>

</xml_diff>